<commit_message>
Remove old document templates and update existing templates for legal documents. Add .gitignore and requirements.txt for project dependencies.
</commit_message>
<xml_diff>
--- a/data/basedatosNatural.xlsx
+++ b/data/basedatosNatural.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-23148" yWindow="-2088" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
@@ -45,10 +45,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -447,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="11.42578125" customWidth="1" style="1" min="1" max="1"/>
@@ -611,30 +614,60 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Ing. Alfonso Reinoso Luis Eduardo</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Pedro Alfonso Pedro Porro</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>1414141441001</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>1414141441</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Jorge Gonzalo Atiencia Gálvez</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ing. Alfonso Reinoso Luis Eduardo</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Pedro Alfonso Pedro Porro</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1414141441001</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1414141441</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>Dr. Jorge Gonzalo Atiencia Gálvez</t>
         </is>

</xml_diff>